<commit_message>
feat: full CRUD users (add/edit/delete), export Excel, REST API microservices, Excel template
</commit_message>
<xml_diff>
--- a/public/template-soal.xlsx
+++ b/public/template-soal.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Template" sheetId="1" r:id="rId1"/>
+    <sheet name="Template Soal" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,141 +397,69 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J6"/>
-  <cols>
-    <col min="1" max="1" width="30.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="20.83203125" customWidth="1"/>
-    <col min="4" max="4" width="20.83203125" customWidth="1"/>
-    <col min="5" max="5" width="20.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.83203125" customWidth="1"/>
-    <col min="7" max="7" width="20.83203125" customWidth="1"/>
-    <col min="8" max="8" width="25.83203125" customWidth="1"/>
-    <col min="9" max="9" width="40.83203125" customWidth="1"/>
-    <col min="10" max="10" width="15.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:I2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Judul Ujian</v>
+        <v>Nama Paket</v>
       </c>
       <c r="B1" t="str">
-        <v>Kategori</v>
+        <v>Pertanyaan</v>
       </c>
       <c r="C1" t="str">
-        <v>Durasi (Menit)</v>
+        <v>A</v>
+      </c>
+      <c r="D1" t="str">
+        <v>B</v>
+      </c>
+      <c r="E1" t="str">
+        <v>C</v>
+      </c>
+      <c r="F1" t="str">
+        <v>D</v>
+      </c>
+      <c r="G1" t="str">
+        <v>E</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Kunci Jawaban</v>
+      </c>
+      <c r="I1" t="str">
+        <v>Pembahasan</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Tryout CPNS 2026 Batch 1</v>
+        <v>Contoh Paket CPNS</v>
       </c>
       <c r="B2" t="str">
-        <v>1</v>
+        <v>Siapakah presiden pertama Indonesia?</v>
       </c>
       <c r="C2" t="str">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>Pertanyaan</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Tipe</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Pilihan A</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Pilihan B</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Pilihan C</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Pilihan D</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Pilihan E</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Jawaban Benar (A/B/C/D/E)</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Pembahasan (Opsional)</v>
-      </c>
-      <c r="J4" t="str">
-        <v>Tingkat Kesulitan</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>Siapa penemu lampu pijar?</v>
-      </c>
-      <c r="B5" t="str">
-        <v>multiple_choice</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Isaac Newton</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Thomas Edison</v>
-      </c>
-      <c r="E5" t="str">
-        <v>Nikola Tesla</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Albert Einstein</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Galileo</v>
-      </c>
-      <c r="H5" t="str">
+        <v>Soeharto</v>
+      </c>
+      <c r="D2" t="str">
+        <v>Soekarno</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Habibie</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Megawati</v>
+      </c>
+      <c r="G2" t="str">
+        <v/>
+      </c>
+      <c r="H2" t="str">
         <v>B</v>
       </c>
-      <c r="I5" t="str">
-        <v>Thomas Edison mematenkan lampu pijar praktis.</v>
-      </c>
-      <c r="J5" t="str">
-        <v>mudah</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>Apa ibu kota Indonesia?</v>
-      </c>
-      <c r="B6" t="str">
-        <v>multiple_choice</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Bandung</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Surabaya</v>
-      </c>
-      <c r="E6" t="str">
-        <v>Semarang</v>
-      </c>
-      <c r="F6" t="str">
-        <v>Jakarta</v>
-      </c>
-      <c r="G6" t="str">
-        <v>Medan</v>
-      </c>
-      <c r="H6" t="str">
-        <v>D</v>
-      </c>
-      <c r="I6" t="str">
-        <v/>
-      </c>
-      <c r="J6" t="str">
-        <v>mudah</v>
+      <c r="I2" t="str">
+        <v>Soekarno adalah presiden pertama Republik Indonesia yang menjabat dari 1945 hingga 1967.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:I2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>